<commit_message>
v5.807 — importatore unico "Caricamento massivo figurine" (sostituisce base + variazioni/change). Riga base se "Figurina base" vuoto (base per Numero o Nome; retro obbligatorio), altrimenti variante/change/errore di quella base; sotto-tipo da Tipo / Tipo di change / Tipo di errore di stampa (mutuamente esclusivi); doppia passata basi-prima; guardia numeri doppi. Nuovo template unico, sezione UI unica; startImportVar dismesso
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YuXK6if3H6iVAZ3AUavow
</commit_message>
<xml_diff>
--- a/templates/template-figurine.xlsx
+++ b/templates/template-figurine.xlsx
@@ -26,9 +26,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -40,7 +40,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004A3F6B"/>
+        <fgColor rgb="FF4A3F6B"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,7 +59,7 @@
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,19 +426,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Serie</t>
@@ -466,10 +470,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Figurina base</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo di change</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo di errore di stampa</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Retro - Categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Retro - Nome</t>
         </is>

</xml_diff>

<commit_message>
v5.812 — semplificazione: nell import unico figurine la colonna errori di stampa si chiama solo "Tipo errore di stampa" (senza di). getCol, template e istruzioni allineati; import retro invariato
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YuXK6if3H6iVAZ3AUavow
</commit_message>
<xml_diff>
--- a/templates/template-figurine.xlsx
+++ b/templates/template-figurine.xlsx
@@ -437,7 +437,7 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
   </cols>
@@ -485,7 +485,7 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Tipo di errore di stampa</t>
+          <t>Tipo errore di stampa</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
v5.814 — import figurine: il retro di riferimento può essere anche un change/errore di stampa di retro. Nuove colonne "Retro - Tipo di change" e "Retro - Tipo errore di stampa"; riconciliazione retro = Categoria+Nome+tipo (Nome resta quello base). Vuote = retro base (retrocompatibile). Template, istruzioni e messaggi aggiornati
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011YuXK6if3H6iVAZ3AUavow
</commit_message>
<xml_diff>
--- a/templates/template-figurine.xlsx
+++ b/templates/template-figurine.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -439,7 +439,9 @@
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,6 +498,16 @@
       <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Retro - Nome</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Tipo di change</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Tipo errore di stampa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v6.372 - i due template dell'import rifatti sulle colonne vere: figurine 15 (era 13), retro 11 (templates/)
</commit_message>
<xml_diff>
--- a/templates/template-figurine.xlsx
+++ b/templates/template-figurine.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figurine" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,12 +27,33 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00606060"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -40,11 +62,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4A3F6B"/>
+        <fgColor rgb="002F3B52"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3B0"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -52,14 +79,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="009AA5B1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -426,88 +466,443 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="8.43" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Serie</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Numero</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sottoserie</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Versione</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Figurina di partenza</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tipologia di change</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tipologia di omaggio</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Tipologia di errore di stampa</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Categoria</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Sottocategoria</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Nome</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Tipo di change</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Tipo di omaggio</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Retro - Tipo di errore</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Template import Figurine — figurinesgorbions.it</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Formato delle colonne: v6.351, meno la Taglia (tolta nella v6.363).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>rifiutato con «colonna mancante»: e' voluto, perche' «Tipo» e «Versione» ora vogliono dire</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>due cose diverse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>COME SI USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>1. Compila il foglio «Figurine»: riga 1 le intestazioni (non toccarle), una riga per figurina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2. Nel sito: Admin -&gt; Foto e import -&gt; Import Figurine. Scegli la serie, carica il file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>3. Le righe con Serie diversa da quella selezionata vengono ignorate, non sono un errore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>4. Le basi si importano prima delle loro varianti: ci pensa la procedura, non serve ordinare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>QUESTO FOGLIO NON VIENE LETTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>L'import legge SOLO il primo foglio del file. Queste istruzioni stanno qui apposta, cosi'</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>non finiscono importate come figurine. Per la stessa ragione nel foglio «Figurine» non c'e'</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>nessuna riga d'esempio: una riga d'esempio in un template da importare diventa un dato vero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>VERSIONE — i sei valori ammessi</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>base  ·  variazione ufficiale  ·  variazione non ufficiale  ·  change  ·  omaggio  ·  errore di stampa</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Scritti cosi', minuscolo o maiuscolo non conta. Un valore diverso ferma la riga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>LE COLONNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Colonna</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>A cosa serve</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>Serie</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Nome completo della serie. Obbligatoria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Numero</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Numero della figurina. Vuoto per le serie senza numero, e per omaggi ed errori di stampa (lo ereditano dalla partenza).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Nome della figurina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Sottoserie</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Taglia</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Figurina base</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo di change</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo errore di stampa</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Solo se la serie ha sottoserie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Versione</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Uno dei sei valori qui sopra. Obbligatoria.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Figurina di partenza</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>SOLO per le versioni non base. Numero della figurina di partenza, o Nome se non ha numero.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Tipologia di change</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Solo con Versione = change. Deve essere una delle tipologie configurate sulla serie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Tipologia di omaggio</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Solo con Versione = omaggio. Idem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Tipologia di errore di stampa</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Solo con Versione = errore di stampa. Idem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>Retro - Categoria</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Categoria del retro da agganciare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Retro - Sottocategoria</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Facoltativa. Serve quando due retro hanno lo stesso Nome in sottocategorie diverse: senza, la riga viene scartata elencando fra quali scegliere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Retro - Nome</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Nome del retro da agganciare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>Retro - Tipo di change</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Retro - Tipo errore di stampa</t>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>Compila solo se il retro da agganciare e' a sua volta un change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Retro - Tipo di omaggio</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Solo se il retro da agganciare e' un omaggio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Retro - Tipo di errore</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Solo se il retro da agganciare e' un errore di stampa.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v6.373 - template import figurine: la colonna Sottoserie passa dopo Serie (templates/)
</commit_message>
<xml_diff>
--- a/templates/template-figurine.xlsx
+++ b/templates/template-figurine.xlsx
@@ -470,9 +470,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
@@ -495,17 +495,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Sottoserie</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Numero</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Nome</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Sottoserie</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -713,7 +713,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>

</xml_diff>